<commit_message>
V1.1.1 - Versión final del proyecto integrador
</commit_message>
<xml_diff>
--- a/reports/comparacion_modelos.xlsx
+++ b/reports/comparacion_modelos.xlsx
@@ -451,45 +451,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>0.9526242452392011</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>0.9538891476478808</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0.9985372988785958</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0.975702715578847</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>0.6715040965191537</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0.9526242452392011</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>0.9526242452392011</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0.9757373929590866</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0.6669534708081185</v>
       </c>
     </row>
     <row r="4">
@@ -499,19 +499,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9944263817928471</v>
+        <v>0.7213190896423595</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9995100440960314</v>
+        <v>0.9594680177327423</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9946367625548513</v>
+        <v>0.7386640663091175</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9970674486803519</v>
+        <v>0.8347107438016529</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9991156872305236</v>
+        <v>0.5722794237148785</v>
       </c>
     </row>
   </sheetData>

</xml_diff>